<commit_message>
Refactor Halloween menu toggle function; add responsive styles for images and create new HTML structure for exercises
</commit_message>
<xml_diff>
--- a/asignaturas/BI/EXCEL/EXAMEN/Naiara_examentipo04.xlsx
+++ b/asignaturas/BI/EXCEL/EXAMEN/Naiara_examentipo04.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAW\asignaturas\BI\EXCEL\EXAMEN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DD61E25-3424-40C1-9C45-D42394655288}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB83853-CC04-403A-93A6-959619FC1BD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23145" yWindow="-90" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{B7422470-46E5-4F40-8B7D-48ACD8540B3C}"/>
+    <workbookView xWindow="-23145" yWindow="-90" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{B7422470-46E5-4F40-8B7D-48ACD8540B3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="11" r:id="rId1"/>
@@ -448,7 +448,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -483,6 +483,8 @@
     <xf numFmtId="9" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -492,9 +494,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2516,19 +2515,19 @@
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="1" t="s">
@@ -2616,11 +2615,11 @@
       <c r="I7" s="2">
         <v>3597</v>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="18">
         <f>SUM(Tablets)</f>
         <v>31215</v>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="18">
         <f>J7*IVA</f>
         <v>6555.15</v>
       </c>
@@ -2647,11 +2646,11 @@
       <c r="I8" s="2">
         <v>5463</v>
       </c>
-      <c r="J8" s="21">
+      <c r="J8" s="18">
         <f>SUM(Tv)</f>
         <v>35425</v>
       </c>
-      <c r="K8" s="21">
+      <c r="K8" s="18">
         <f>J8*IVA</f>
         <v>7439.25</v>
       </c>
@@ -2678,11 +2677,11 @@
       <c r="I9" s="2">
         <v>1185</v>
       </c>
-      <c r="J9" s="21">
+      <c r="J9" s="18">
         <f>SUM(Ordenadores)</f>
         <v>26882</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="18">
         <f>J9*IVA</f>
         <v>5645.2199999999993</v>
       </c>
@@ -2709,11 +2708,11 @@
       <c r="I10" s="2">
         <v>3398</v>
       </c>
-      <c r="J10" s="21">
+      <c r="J10" s="18">
         <f>SUM(Ratones)</f>
         <v>29850</v>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="18">
         <f>J10*IVA</f>
         <v>6268.5</v>
       </c>
@@ -2740,55 +2739,55 @@
       <c r="I11" s="2">
         <v>1956</v>
       </c>
-      <c r="J11" s="21">
+      <c r="J11" s="18">
         <f>SUM(Pantallas)</f>
         <v>20073</v>
       </c>
-      <c r="K11" s="21">
+      <c r="K11" s="18">
         <f>J11*IVA</f>
         <v>4215.33</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="21">
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="18">
         <f>F10</f>
         <v>5634</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15">
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="21">
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="18">
         <f>SUM(Julio,Agosto,Septiembre)</f>
         <v>78203</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15">
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="21">
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="18">
         <f>SUM(Tv,Tablets)</f>
         <v>66640</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="15">
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="21">
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="18">
         <f>SUM(Iva_Total)</f>
         <v>30123.449999999997</v>
       </c>
@@ -2832,7 +2831,11 @@
         <v>2</v>
       </c>
       <c r="D7" s="16" t="str">
-        <f t="shared" ref="D7:D8" si="0">_xlfn.IFS((ISERR(C7=0)),C7&lt;1,C7&lt;3,"Bebe",C7&lt;10,"Niño",C7&lt;15,"Preadolescente",C7&lt;18,"Adolescente",C7&lt;49,"Joven",C7&lt;50,"Adulto",C7&lt;81,"mayor",C7&lt;100,"mayor")</f>
+        <f>_xlfn.IFS((ISERR(C7=0)),C7&lt;1,C7&lt;3,"Bebe",C7&lt;10,"Niño",C7&lt;15,"Preadolescente",C7&lt;18,"Adolescente",C7&lt;49,"Joven",C7&lt;50,"Adulto",C7&lt;81,"mayor",C7&lt;100,"mayor")</f>
+        <v>Bebe</v>
+      </c>
+      <c r="F7" t="str">
+        <f>IF(C7&lt;=3,"Bebe",IF(C7&lt;=10,"Niño",IF(C7&lt;=13,"Preadolescente",IF(C7&lt;=18,"Adolescente",IF(C7&lt;=50,"Joven",IF(C7&lt;=65,"Adulto",IF(C7&lt;=80,"Mayor",IF(C7&lt;=100,"Anciano"))))))))</f>
         <v>Bebe</v>
       </c>
     </row>
@@ -2841,7 +2844,11 @@
         <v>12</v>
       </c>
       <c r="D8" s="16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D7:D8" si="0">_xlfn.IFS((ISERR(C8=0)),C8&lt;1,C8&lt;3,"Bebe",C8&lt;10,"Niño",C8&lt;15,"Preadolescente",C8&lt;18,"Adolescente",C8&lt;49,"Joven",C8&lt;50,"Adulto",C8&lt;81,"mayor",C8&lt;100,"mayor")</f>
+        <v>Preadolescente</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" ref="F8:F11" si="1">IF(C8&lt;=3,"Bebe",IF(C8&lt;=10,"Niño",IF(C8&lt;=13,"Preadolescente",IF(C8&lt;=18,"Adolescente",IF(C8&lt;=50,"Joven",IF(C8&lt;=65,"Adulto",IF(C8&lt;=80,"Mayor",IF(C8&lt;=100,"Anciano"))))))))</f>
         <v>Preadolescente</v>
       </c>
     </row>
@@ -2853,14 +2860,22 @@
         <f>_xlfn.IFS((ISERR(C9=0)),C9&lt;1,C9&lt;3,"Bebe",C9&lt;10,"Niño",C9&lt;15,"Preadolescente",C9&lt;18,"Adolescente",C9&lt;49,"Joven",C9&lt;50,"Adulto",C9&lt;81,"mayor",C9&lt;100,"mayor")</f>
         <v>Joven</v>
       </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v>Joven</v>
+      </c>
     </row>
     <row r="10" spans="3:6">
       <c r="C10" s="1">
         <v>65</v>
       </c>
       <c r="D10" s="16" t="str">
-        <f t="shared" ref="D10:D11" si="1">_xlfn.IFS((ISERR(C10=0)),C10&lt;1,C10&lt;3,"Bebe",C10&lt;10,"Niño",C10&lt;15,"Preadolescente",C10&lt;18,"Adolescente",C10&lt;49,"Joven",C10&lt;50,"Adulto",C10&lt;81,"mayor",C10&lt;100,"mayor")</f>
+        <f t="shared" ref="D10" si="2">_xlfn.IFS((ISERR(C10=0)),C10&lt;1,C10&lt;3,"Bebe",C10&lt;10,"Niño",C10&lt;15,"Preadolescente",C10&lt;18,"Adolescente",C10&lt;49,"Joven",C10&lt;50,"Adulto",C10&lt;81,"mayor",C10&lt;100,"mayor")</f>
         <v>mayor</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>Adulto</v>
       </c>
     </row>
     <row r="11" spans="3:6">
@@ -2871,71 +2886,74 @@
         <f>_xlfn.IFS((ISERR(C11=0)),C11&lt;1,C11&lt;3,"Bebe",C11&lt;10,"Niño",C11&lt;15,"Preadolescente",C11&lt;18,"Adolescente",C11&lt;49,"Joven",C11&lt;50,"Adulto",C11&lt;81,"mayor",C11&lt;100,"mayor")</f>
         <v>mayor</v>
       </c>
-      <c r="F11" s="23"/>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v>Anciano</v>
+      </c>
     </row>
     <row r="14" spans="3:6">
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="3:6">
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" spans="3:6">
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="17" spans="3:6">
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
     </row>
     <row r="18" spans="3:6">
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" spans="3:6">
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" spans="3:6">
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
     </row>
     <row r="21" spans="3:6">
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3004,15 +3022,15 @@
       <c r="E7" s="8">
         <v>100</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="19">
         <f>D7*E7</f>
         <v>1500</v>
       </c>
-      <c r="G7" s="21" t="b">
+      <c r="G7" s="18" t="b">
         <f>IF(C7="NORTE",AND(F7&gt;900),"100 €")</f>
         <v>1</v>
       </c>
-      <c r="H7" s="21"/>
+      <c r="H7" s="18"/>
     </row>
     <row r="8" spans="2:8" ht="15">
       <c r="B8" s="8" t="s">
@@ -3027,15 +3045,15 @@
       <c r="E8" s="8">
         <v>250</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="19">
         <f t="shared" ref="F8:F14" si="0">D8*E8</f>
         <v>5000</v>
       </c>
-      <c r="G8" s="21" t="str">
+      <c r="G8" s="18" t="str">
         <f t="shared" ref="G8:G14" si="1">IF(C8="NORTE",AND(F8&gt;900),"100 €")</f>
         <v>100 €</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" spans="2:8" ht="15">
       <c r="B9" s="8" t="s">
@@ -3050,15 +3068,15 @@
       <c r="E9" s="8">
         <v>100</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="19">
         <f t="shared" si="0"/>
         <v>4600</v>
       </c>
-      <c r="G9" s="21" t="str">
+      <c r="G9" s="18" t="str">
         <f t="shared" si="1"/>
         <v>100 €</v>
       </c>
-      <c r="H9" s="21"/>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="2:8" ht="15">
       <c r="B10" s="8" t="s">
@@ -3073,15 +3091,15 @@
       <c r="E10" s="8">
         <v>150</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="19">
         <f t="shared" si="0"/>
         <v>4800</v>
       </c>
-      <c r="G10" s="21" t="b">
+      <c r="G10" s="18" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H10" s="21"/>
+      <c r="H10" s="18"/>
     </row>
     <row r="11" spans="2:8" ht="15">
       <c r="B11" s="8" t="s">
@@ -3096,15 +3114,15 @@
       <c r="E11" s="8">
         <v>300</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="19">
         <f t="shared" si="0"/>
         <v>5400</v>
       </c>
-      <c r="G11" s="21" t="str">
+      <c r="G11" s="18" t="str">
         <f t="shared" si="1"/>
         <v>100 €</v>
       </c>
-      <c r="H11" s="21"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" spans="2:8" ht="15">
       <c r="B12" s="8" t="s">
@@ -3119,15 +3137,15 @@
       <c r="E12" s="8">
         <v>25</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="19">
         <f t="shared" si="0"/>
         <v>175</v>
       </c>
-      <c r="G12" s="21" t="b">
+      <c r="G12" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="2:8" ht="15">
       <c r="B13" s="8" t="s">
@@ -3142,15 +3160,15 @@
       <c r="E13" s="8">
         <v>250</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="19">
         <f t="shared" si="0"/>
         <v>5750</v>
       </c>
-      <c r="G13" s="21" t="str">
+      <c r="G13" s="18" t="str">
         <f t="shared" si="1"/>
         <v>100 €</v>
       </c>
-      <c r="H13" s="21"/>
+      <c r="H13" s="18"/>
     </row>
     <row r="14" spans="2:8" ht="15">
       <c r="B14" s="8" t="s">
@@ -3165,15 +3183,15 @@
       <c r="E14" s="8">
         <v>25</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="19">
         <f t="shared" si="0"/>
         <v>175</v>
       </c>
-      <c r="G14" s="21" t="b">
+      <c r="G14" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H14" s="21"/>
+      <c r="H14" s="18"/>
     </row>
     <row r="16" spans="2:8" ht="15">
       <c r="B16" s="9"/>

</xml_diff>

<commit_message>
Add connection scripts, logout functionality, and update API references; enhance layout and styles for exam projects
</commit_message>
<xml_diff>
--- a/asignaturas/BI/EXCEL/EXAMEN/Naiara_examentipo04.xlsx
+++ b/asignaturas/BI/EXCEL/EXAMEN/Naiara_examentipo04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAW\asignaturas\BI\EXCEL\EXAMEN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB83853-CC04-403A-93A6-959619FC1BD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9937863D-6358-4DDC-856A-442F718CE902}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23145" yWindow="-90" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{B7422470-46E5-4F40-8B7D-48ACD8540B3C}"/>
+    <workbookView minimized="1" xWindow="-23145" yWindow="-90" windowWidth="23250" windowHeight="12450" activeTab="4" xr2:uid="{B7422470-46E5-4F40-8B7D-48ACD8540B3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="11" r:id="rId1"/>
@@ -27,6 +27,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Ej5 '!$A$6:$E$40</definedName>
     <definedName name="Agosto">'Ej1'!$E$6:$E$11</definedName>
+    <definedName name="AUMENTO">'Ej4'!$F$6:$F$14</definedName>
     <definedName name="Diciembre">'Ej1'!$I$6:$I$11</definedName>
     <definedName name="ingresos2017">'[1]Ejercicio conjunto'!$F$7:$F$19</definedName>
     <definedName name="IVA">'Ej1'!$L$6</definedName>
@@ -41,6 +42,9 @@
     <definedName name="Tablets">'Ej1'!$C$7:$I$7</definedName>
     <definedName name="Total">'Ej1'!$J$6:$J$11</definedName>
     <definedName name="Tv">'Ej1'!$C$8:$I$8</definedName>
+    <definedName name="UNIDADES_ASIGNADAS">'Ej4'!$D$6:$D$14</definedName>
+    <definedName name="VENDEDOR" localSheetId="4">'Ej4'!$C$6:$C$14</definedName>
+    <definedName name="ZONA" localSheetId="4">'Ej4'!$E$6:$E$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="93">
   <si>
     <t>Total</t>
   </si>
@@ -311,6 +315,27 @@
   </si>
   <si>
     <t>La empresa decide que para cada fila, solo se pueden poner % de aumento si las unidades asignadas son mayor a 9 y la zona es norte o superiores a 40  y la zona es sur.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B  </t>
+  </si>
+  <si>
+    <t>Juan</t>
+  </si>
+  <si>
+    <t>VALENTIN</t>
+  </si>
+  <si>
+    <t>ENTREGADA</t>
+  </si>
+  <si>
+    <t>NO ENTREGADA</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Kira</t>
   </si>
 </sst>
 </file>
@@ -2616,11 +2641,11 @@
         <v>3597</v>
       </c>
       <c r="J7" s="18">
-        <f>SUM(Tablets)</f>
+        <f ca="1">SUM(INDIRECT(C7))</f>
         <v>31215</v>
       </c>
       <c r="K7" s="18">
-        <f>J7*IVA</f>
+        <f ca="1">J7*IVA</f>
         <v>6555.15</v>
       </c>
     </row>
@@ -2647,11 +2672,11 @@
         <v>5463</v>
       </c>
       <c r="J8" s="18">
-        <f>SUM(Tv)</f>
+        <f t="shared" ref="J8:J11" ca="1" si="0">SUM(INDIRECT(C8))</f>
         <v>35425</v>
       </c>
       <c r="K8" s="18">
-        <f>J8*IVA</f>
+        <f ca="1">J8*IVA</f>
         <v>7439.25</v>
       </c>
     </row>
@@ -2678,11 +2703,11 @@
         <v>1185</v>
       </c>
       <c r="J9" s="18">
-        <f>SUM(Ordenadores)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>26882</v>
       </c>
       <c r="K9" s="18">
-        <f>J9*IVA</f>
+        <f ca="1">J9*IVA</f>
         <v>5645.2199999999993</v>
       </c>
     </row>
@@ -2709,11 +2734,11 @@
         <v>3398</v>
       </c>
       <c r="J10" s="18">
-        <f>SUM(Ratones)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>29850</v>
       </c>
       <c r="K10" s="18">
-        <f>J10*IVA</f>
+        <f ca="1">J10*IVA</f>
         <v>6268.5</v>
       </c>
     </row>
@@ -2740,11 +2765,11 @@
         <v>1956</v>
       </c>
       <c r="J11" s="18">
-        <f>SUM(Pantallas)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>20073</v>
       </c>
       <c r="K11" s="18">
-        <f>J11*IVA</f>
+        <f ca="1">J11*IVA</f>
         <v>4215.33</v>
       </c>
     </row>
@@ -2788,7 +2813,7 @@
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
       <c r="E20" s="18">
-        <f>SUM(Iva_Total)</f>
+        <f ca="1">SUM(Iva_Total)</f>
         <v>30123.449999999997</v>
       </c>
     </row>
@@ -2835,7 +2860,7 @@
         <v>Bebe</v>
       </c>
       <c r="F7" t="str">
-        <f>IF(C7&lt;=3,"Bebe",IF(C7&lt;=10,"Niño",IF(C7&lt;=13,"Preadolescente",IF(C7&lt;=18,"Adolescente",IF(C7&lt;=50,"Joven",IF(C7&lt;=65,"Adulto",IF(C7&lt;=80,"Mayor",IF(C7&lt;=100,"Anciano"))))))))</f>
+        <f>IF(C7&lt;=3,"Bebe",IF(C7&lt;=10,"Niño",IF(C7&lt;=13,"Preadolescente",IF(C7&lt;=18,"Adolescente",IF(C7&lt;=50,"Joven",IF(C7&lt;=67,"Adulto",IF(C7&lt;=81,"Mayor",IF(C7&lt;=100,"Anciano"))))))))</f>
         <v>Bebe</v>
       </c>
     </row>
@@ -2844,7 +2869,7 @@
         <v>12</v>
       </c>
       <c r="D8" s="16" t="str">
-        <f t="shared" ref="D7:D8" si="0">_xlfn.IFS((ISERR(C8=0)),C8&lt;1,C8&lt;3,"Bebe",C8&lt;10,"Niño",C8&lt;15,"Preadolescente",C8&lt;18,"Adolescente",C8&lt;49,"Joven",C8&lt;50,"Adulto",C8&lt;81,"mayor",C8&lt;100,"mayor")</f>
+        <f t="shared" ref="D8" si="0">_xlfn.IFS((ISERR(C8=0)),C8&lt;1,C8&lt;3,"Bebe",C8&lt;10,"Niño",C8&lt;15,"Preadolescente",C8&lt;18,"Adolescente",C8&lt;49,"Joven",C8&lt;50,"Adulto",C8&lt;81,"mayor",C8&lt;100,"mayor")</f>
         <v>Preadolescente</v>
       </c>
       <c r="F8" t="str">
@@ -3026,9 +3051,8 @@
         <f>D7*E7</f>
         <v>1500</v>
       </c>
-      <c r="G7" s="18" t="b">
-        <f>IF(C7="NORTE",AND(F7&gt;900),"100 €")</f>
-        <v>1</v>
+      <c r="G7" s="18" t="s">
+        <v>86</v>
       </c>
       <c r="H7" s="18"/>
     </row>
@@ -3205,7 +3229,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06278CF0-F8AC-4B2B-B625-078485695FFC}">
-  <dimension ref="C6:J27"/>
+  <dimension ref="C6:J28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="3" max="3" width="15.125" bestFit="1" customWidth="1"/>
@@ -3233,8 +3257,12 @@
       </c>
     </row>
     <row r="7" spans="3:10">
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="C7" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="1">
+        <v>48</v>
+      </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="H7" t="s">
@@ -3242,7 +3270,9 @@
       </c>
     </row>
     <row r="8" spans="3:10">
-      <c r="C8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -3251,7 +3281,9 @@
       </c>
     </row>
     <row r="9" spans="3:10">
-      <c r="C9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -3260,83 +3292,117 @@
       </c>
     </row>
     <row r="10" spans="3:10">
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="3:10">
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="3:10">
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="3:10">
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="3:10">
-      <c r="J14" s="13"/>
-    </row>
-    <row r="17" spans="3:8" ht="15">
-      <c r="C17" s="4" t="s">
+      <c r="C14" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="3:10">
+      <c r="J15" s="13"/>
+    </row>
+    <row r="18" spans="3:8" ht="15">
+      <c r="C18" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="3:8">
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="H18" t="s">
+    <row r="19" spans="3:8">
+      <c r="C19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="1">
+        <v>5</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="1">
+        <v>5</v>
+      </c>
+      <c r="H19" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="3:8">
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="H19" t="s">
+    <row r="20" spans="3:8">
+      <c r="C20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="1">
+        <v>9</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="1">
+        <v>9</v>
+      </c>
+      <c r="H20" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="3:8">
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="H20" t="s">
+    <row r="21" spans="3:8">
+      <c r="C21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="H21" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="21" spans="3:8">
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
     </row>
     <row r="22" spans="3:8">
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="E22" s="1" t="s">
+        <v>89</v>
+      </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="3:8">
@@ -3351,26 +3417,42 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
     </row>
-    <row r="27" spans="3:8">
-      <c r="H27" t="s">
+    <row r="25" spans="3:8">
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="28" spans="3:8">
+      <c r="H28" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
-  <dataValidations count="4">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="No puedes tener menos de 0 de stock" sqref="F18:F24" xr:uid="{705E55E9-114A-4007-8C8F-A562BAE17C88}">
-      <formula1>F18&gt;=0</formula1>
+  <dataValidations xWindow="616" yWindow="726" count="7">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Nombre" prompt="Debes introducir un nombre" sqref="C19:C25" xr:uid="{FDDD23E1-1C51-430A-817B-E508D601878B}">
+      <formula1>COUNTIF($C$19:$C$25,C19) = 1</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C18:C24" xr:uid="{FDDD23E1-1C51-430A-817B-E508D601878B}">
-      <formula1>COUNTIF($C$18:$C$24,C18) = 1</formula1>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="No corresponde con las zonas asignadas" promptTitle="Zona" prompt="Debes introducir zona &quot;NORTE&quot; o &quot;SUR&quot;" sqref="E7:E14" xr:uid="{4DF7F5DD-B7AC-49A7-81C0-1AA7BAE4F8DC}">
+      <formula1>"SUR,NORTE"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Debe ser un teléfono móvil que comience por 6 o un fijo que comience por 9" sqref="E7:E13" xr:uid="{4DF7F5DD-B7AC-49A7-81C0-1AA7BAE4F8DC}">
-      <formula1>OR(AND(E7&gt;600000000,E7&lt;699999999),AND(E7&gt;900000000,E7&lt;999999999))</formula1>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C7:C14" xr:uid="{8177FACC-4C00-44DC-B8DB-B755C55A5983}">
+      <formula1>"VALENTIN,SERGIO,ANTONIO,DAMIAN"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Solo se permiten edades entre 18 y 70 años" sqref="D7:D13" xr:uid="{DF2D9F0B-57E7-430D-928E-C0E86DA41779}">
-      <formula1>18</formula1>
-      <formula2>70</formula2>
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" errorTitle="Aprobado" error="Para aprobar debes tener más de un 4,5" promptTitle="Nota" prompt="Debes introdcuir una nota" sqref="F19:F25" xr:uid="{8C8CA337-3B97-4BF5-9B21-BBAFFA87666B}">
+      <formula1>5</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="list" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Tarea" error="No coincide con lo proporcionado" promptTitle="Tarea" prompt="Debes introducir si está &quot;ENTEGRADA&quot; o &quot;NO ENTREGADA&quot;" sqref="E19:E25" xr:uid="{5BC30AE4-FE07-4B3B-AFF3-092B85C857F4}">
+      <formula1>"ENTREGADA,NO ENTREGADA"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" errorTitle="Nota" error="No puede ser menor a 1 ni mayor a 10" promptTitle="Nota" prompt="Debes introducir una nota entre el 1 al 10" sqref="D19:D25" xr:uid="{5882B663-538A-43C6-9603-CCB0BACF488D}">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" errorTitle="Unidad" error="No se le pueden asignar más de 70 unidades" promptTitle="Unidad" prompt="Introduce una unidad" sqref="D7:D14" xr:uid="{D07EBE79-6716-45AF-B59C-A77D19393662}">
+      <formula1>D7:E7&lt;70</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>